<commit_message>
adding find and replace
</commit_message>
<xml_diff>
--- a/Excel/27_Notes_and_Comments/Pinterest_Notes_and_Comments.xlsx
+++ b/Excel/27_Notes_and_Comments/Pinterest_Notes_and_Comments.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Pinterest-Analytics-Project\Excel\27_Notes_and_Comments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B7F8B93-BC27-4145-B251-5EFA7B7E2A9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA586D3B-6310-4C65-9F1C-9CD5848290FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D2A27962-3810-4A74-AC6E-986E11F82A8E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{D2A27962-3810-4A74-AC6E-986E11F82A8E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Pin_Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Notes_practice" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,9 +36,141 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Rekha Musale</author>
+    <author>tc={616C1726-6843-45F1-BCFF-971897B1A203}</author>
+  </authors>
+  <commentList>
+    <comment ref="C2" authorId="0" shapeId="0" xr:uid="{8F0C2C6D-3704-472E-AEA2-9DE16361521B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rekha Musale:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Impressions recorded for the Wooden Knife Holder Pinterest pin in the sample dataset.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D3" authorId="1" shapeId="0" xr:uid="{616C1726-6843-45F1-BCFF-971897B1A203}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Handbag Fashion has 2 engagements. Review this pin's performance when comparing fashion content.
+</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Rekha Musale</author>
+    <author>tc={92E1DC81-BFAB-4631-969D-B6CE2FC6F365}</author>
+  </authors>
+  <commentList>
+    <comment ref="C2" authorId="0" shapeId="0" xr:uid="{01C2A30C-7D37-4E98-B724-8A6DD316AA0D}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rekha Musale:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Impressions recorded for the Wooden Knife Holder Pinterest pin in the sample dataset.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D3" authorId="1" shapeId="0" xr:uid="{92E1DC81-BFAB-4631-969D-B6CE2FC6F365}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Handbag Fashion has 2 engagements. Review this pin's performance when comparing fashion content.
+</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="13">
+  <si>
+    <t>PinName</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Impressions</t>
+  </si>
+  <si>
+    <t>Engagement</t>
+  </si>
+  <si>
+    <t>Wooden-Knife-Holder</t>
+  </si>
+  <si>
+    <t>Kitchen</t>
+  </si>
+  <si>
+    <t>Handbag-Fashion</t>
+  </si>
+  <si>
+    <t>Fashion</t>
+  </si>
+  <si>
+    <t>Beauty-Self-Care</t>
+  </si>
+  <si>
+    <t>Beauty</t>
+  </si>
+  <si>
+    <t>Kitchen-Storage</t>
+  </si>
+  <si>
+    <t>Home-Decor-Ideas</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -45,16 +178,41 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -62,12 +220,174 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -83,6 +403,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Rekha Musale" id="{D8AEE39C-3CB7-4373-82AA-72C8184793FD}" userId="afea116efc88aa0e" providerId="Windows Live"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -400,11 +726,222 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="D3" dT="2026-10-27T13:52:17.10" personId="{D8AEE39C-3CB7-4373-82AA-72C8184793FD}" id="{616C1726-6843-45F1-BCFF-971897B1A203}">
+    <text xml:space="preserve">Handbag Fashion has 2 engagements. Review this pin's performance when comparing fashion content.
+</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="D3" dT="2026-10-27T13:52:17.10" personId="{D8AEE39C-3CB7-4373-82AA-72C8184793FD}" id="{92E1DC81-BFAB-4631-969D-B6CE2FC6F365}">
+    <text xml:space="preserve">Handbag Fashion has 2 engagements. Review this pin's performance when comparing fashion content.
+</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0034629B-15D4-43A3-9EF4-0BDB12250DDA}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0034629B-15D4-43A3-9EF4-0BDB12250DDA}">
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1">
+        <v>214</v>
+      </c>
+      <c r="D2" s="6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1">
+        <v>45</v>
+      </c>
+      <c r="D3" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1">
+        <v>57</v>
+      </c>
+      <c r="D4" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="1">
+        <v>76</v>
+      </c>
+      <c r="D5" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="8">
+        <v>41</v>
+      </c>
+      <c r="D6" s="9">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFF5B729-812B-4F11-89E7-431EE4A82D74}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1">
+        <v>214</v>
+      </c>
+      <c r="D2" s="6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1">
+        <v>45</v>
+      </c>
+      <c r="D3" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1">
+        <v>57</v>
+      </c>
+      <c r="D4" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="1">
+        <v>76</v>
+      </c>
+      <c r="D5" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="8">
+        <v>41</v>
+      </c>
+      <c r="D6" s="9">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>